<commit_message>
fix(car-spin): move ultrasonic pins to GPIO3 and GPIO46
</commit_message>
<xml_diff>
--- a/引脚对应表2.xlsx
+++ b/引脚对应表2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\11清华云盘资料库\大二\电设\vscode-esp32s3_testcode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D36E83A-2524-47B2-82EF-DC623A80EDD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53F7139B-932D-400F-805D-0DA0875B2A0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="21806" windowHeight="13886" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="51" yWindow="189" windowWidth="10483" windowHeight="12325" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -175,13 +175,7 @@
     <t>GND</t>
   </si>
   <si>
-    <t>GPIO40</t>
-  </si>
-  <si>
     <t>Trig(接收高电平后触发测距信号)</t>
-  </si>
-  <si>
-    <t>GPIO39</t>
   </si>
   <si>
     <t>Echo(高电平持续时间正比于超声波往返时间，回响信号输出)</t>
@@ -255,6 +249,14 @@
   </si>
   <si>
     <t>GPIO43</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>GPIO3</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>GPIO46</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -900,20 +902,20 @@
       <c r="C30" s="3"/>
     </row>
     <row r="31" spans="1:3" ht="16.3" x14ac:dyDescent="0.3">
-      <c r="A31" s="5" t="s">
+      <c r="A31" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="B31" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="C31" s="5"/>
+    </row>
+    <row r="32" spans="1:3" ht="16.3" x14ac:dyDescent="0.3">
+      <c r="A32" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="B32" s="4" t="s">
         <v>46</v>
-      </c>
-      <c r="C31" s="5"/>
-    </row>
-    <row r="32" spans="1:3" ht="16.3" x14ac:dyDescent="0.3">
-      <c r="A32" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>48</v>
       </c>
       <c r="C32" s="3"/>
     </row>
@@ -927,7 +929,7 @@
         <v>0</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C34" s="3"/>
     </row>
@@ -942,19 +944,19 @@
     </row>
     <row r="36" spans="1:3" ht="16.3" x14ac:dyDescent="0.3">
       <c r="A36" s="10" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C36" s="3"/>
     </row>
     <row r="37" spans="1:3" ht="16.3" x14ac:dyDescent="0.3">
       <c r="A37" s="11" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C37" s="5"/>
     </row>
@@ -968,7 +970,7 @@
         <v>0</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C39" s="5"/>
     </row>
@@ -990,46 +992,46 @@
     </row>
     <row r="42" spans="1:3" ht="16.3" x14ac:dyDescent="0.3">
       <c r="A42" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C42" s="3"/>
     </row>
     <row r="43" spans="1:3" ht="16.3" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C43" s="5"/>
     </row>
     <row r="44" spans="1:3" ht="16.3" x14ac:dyDescent="0.3">
       <c r="A44" s="3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C44" s="3"/>
     </row>
     <row r="45" spans="1:3" ht="16.3" x14ac:dyDescent="0.3">
       <c r="A45" s="5" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C45" s="5"/>
     </row>
     <row r="46" spans="1:3" ht="16.3" x14ac:dyDescent="0.3">
       <c r="A46" s="3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C46" s="3"/>
     </row>
@@ -1043,7 +1045,7 @@
         <v>0</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C48" s="3"/>
     </row>
@@ -1059,7 +1061,7 @@
     <row r="50" spans="1:3" ht="16.3" x14ac:dyDescent="0.3">
       <c r="A50" s="3"/>
       <c r="B50" s="4" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C50" s="3"/>
     </row>
@@ -1073,35 +1075,35 @@
         <v>0</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C52" s="3"/>
     </row>
     <row r="53" spans="1:3" ht="16.3" x14ac:dyDescent="0.3">
       <c r="A53" s="5"/>
       <c r="B53" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C53" s="5"/>
     </row>
     <row r="54" spans="1:3" ht="16.3" x14ac:dyDescent="0.3">
       <c r="A54" s="3"/>
       <c r="B54" s="3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C54" s="3"/>
     </row>
     <row r="55" spans="1:3" ht="16.3" x14ac:dyDescent="0.3">
       <c r="A55" s="5"/>
       <c r="B55" s="5" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C55" s="5"/>
     </row>
     <row r="56" spans="1:3" ht="16.3" x14ac:dyDescent="0.3">
       <c r="A56" s="3"/>
       <c r="B56" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C56" s="3"/>
     </row>

</xml_diff>